<commit_message>
fixed the parental-daughter analysis. wrote the wrong variable when filtering for the dataframe
</commit_message>
<xml_diff>
--- a/data/analysisTable.xlsx
+++ b/data/analysisTable.xlsx
@@ -1015,7 +1015,7 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>1</v>
+        <v>0.9768441138249091</v>
       </c>
     </row>
     <row r="19">
@@ -1046,7 +1046,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>1</v>
+        <v>0.8013646728044529</v>
       </c>
     </row>
     <row r="20">
@@ -1651,7 +1651,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>1</v>
+        <v>0.9768441138249091</v>
       </c>
     </row>
     <row r="41">
@@ -1682,7 +1682,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>1</v>
+        <v>0.8013646728044529</v>
       </c>
     </row>
     <row r="42">
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="K62" t="n">
-        <v>1</v>
+        <v>0.9768441138249091</v>
       </c>
     </row>
     <row r="63">
@@ -2318,7 +2318,7 @@
         </is>
       </c>
       <c r="K63" t="n">
-        <v>1</v>
+        <v>0.8013646728044529</v>
       </c>
     </row>
     <row r="64">
@@ -2984,7 +2984,7 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>1</v>
+        <v>0.1643488033433622</v>
       </c>
     </row>
     <row r="19">
@@ -3015,7 +3015,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>1</v>
+        <v>1.021692979439843e-05</v>
       </c>
     </row>
     <row r="20">
@@ -3620,7 +3620,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>1</v>
+        <v>0.1643488033433622</v>
       </c>
     </row>
     <row r="41">
@@ -3651,7 +3651,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>1</v>
+        <v>1.021692979439843e-05</v>
       </c>
     </row>
     <row r="42">
@@ -4256,7 +4256,7 @@
         </is>
       </c>
       <c r="K62" t="n">
-        <v>1</v>
+        <v>0.1643488033433622</v>
       </c>
     </row>
     <row r="63">
@@ -4287,7 +4287,7 @@
         </is>
       </c>
       <c r="K63" t="n">
-        <v>1</v>
+        <v>1.021692979439843e-05</v>
       </c>
     </row>
     <row r="64">
@@ -4953,7 +4953,7 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>1</v>
+        <v>0.01410870956425703</v>
       </c>
     </row>
     <row r="19">
@@ -4984,7 +4984,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>1</v>
+        <v>0.001090740331685134</v>
       </c>
     </row>
     <row r="20">
@@ -5589,7 +5589,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>1</v>
+        <v>0.01410870956425703</v>
       </c>
     </row>
     <row r="41">
@@ -5620,7 +5620,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>1</v>
+        <v>0.001090740331685134</v>
       </c>
     </row>
     <row r="42">
@@ -6225,7 +6225,7 @@
         </is>
       </c>
       <c r="K62" t="n">
-        <v>1</v>
+        <v>0.01410870956425703</v>
       </c>
     </row>
     <row r="63">
@@ -6256,7 +6256,7 @@
         </is>
       </c>
       <c r="K63" t="n">
-        <v>1</v>
+        <v>0.001090740331685134</v>
       </c>
     </row>
     <row r="64">
@@ -6922,7 +6922,7 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>1</v>
+        <v>0.1840751043955202</v>
       </c>
     </row>
     <row r="19">
@@ -6953,7 +6953,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>1</v>
+        <v>0.0132086937487541</v>
       </c>
     </row>
     <row r="20">
@@ -7558,7 +7558,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>1</v>
+        <v>0.1840751043955202</v>
       </c>
     </row>
     <row r="41">
@@ -7589,7 +7589,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>1</v>
+        <v>0.0132086937487541</v>
       </c>
     </row>
     <row r="42">
@@ -8194,7 +8194,7 @@
         </is>
       </c>
       <c r="K62" t="n">
-        <v>1</v>
+        <v>0.1840751043955202</v>
       </c>
     </row>
     <row r="63">
@@ -8225,7 +8225,7 @@
         </is>
       </c>
       <c r="K63" t="n">
-        <v>1</v>
+        <v>0.0132086937487541</v>
       </c>
     </row>
     <row r="64">
@@ -8891,7 +8891,7 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>1</v>
+        <v>0.00315367822989782</v>
       </c>
     </row>
     <row r="19">
@@ -8922,7 +8922,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>1</v>
+        <v>2.056424389735719e-09</v>
       </c>
     </row>
     <row r="20">
@@ -9527,7 +9527,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>1</v>
+        <v>0.00315367822989782</v>
       </c>
     </row>
     <row r="41">
@@ -9558,7 +9558,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>1</v>
+        <v>2.056424389735719e-09</v>
       </c>
     </row>
     <row r="42">
@@ -10163,7 +10163,7 @@
         </is>
       </c>
       <c r="K62" t="n">
-        <v>1</v>
+        <v>0.00315367822989782</v>
       </c>
     </row>
     <row r="63">
@@ -10194,7 +10194,7 @@
         </is>
       </c>
       <c r="K63" t="n">
-        <v>1</v>
+        <v>2.056424389735719e-09</v>
       </c>
     </row>
     <row r="64">

</xml_diff>

<commit_message>
removed genes without distances and redid the parental-daughter identification
</commit_message>
<xml_diff>
--- a/data/analysisTable.xlsx
+++ b/data/analysisTable.xlsx
@@ -1018,7 +1018,7 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>0.9768441138249091</v>
+        <v>0.9862180395120353</v>
       </c>
     </row>
     <row r="19">
@@ -1028,13 +1028,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>123</v>
+        <v>43</v>
       </c>
       <c r="C19" t="n">
-        <v>36.64805110021803</v>
+        <v>81.10617979073703</v>
       </c>
       <c r="D19" t="n">
-        <v>521.9703966813282</v>
+        <v>1272.711691675059</v>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
@@ -1049,7 +1049,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>0.8013646728044529</v>
+        <v>0.8558998054368265</v>
       </c>
     </row>
     <row r="20">
@@ -1059,13 +1059,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>121</v>
+        <v>43</v>
       </c>
       <c r="C20" t="n">
-        <v>33.99453807883257</v>
+        <v>87.69343443488347</v>
       </c>
       <c r="D20" t="n">
-        <v>637.875054679287</v>
+        <v>1557.046404031143</v>
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
@@ -1077,13 +1077,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>224</v>
+        <v>65</v>
       </c>
       <c r="C21" t="n">
-        <v>22.04535114126693</v>
+        <v>42.05024144982589</v>
       </c>
       <c r="D21" t="n">
-        <v>283.0514422036969</v>
+        <v>305.2020155903968</v>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
@@ -1095,13 +1095,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>213</v>
+        <v>65</v>
       </c>
       <c r="C22" t="n">
-        <v>16.67727831298509</v>
+        <v>39.91526560386543</v>
       </c>
       <c r="D22" t="n">
-        <v>362.7401690272649</v>
+        <v>627.511222150869</v>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
@@ -1648,7 +1648,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>0.1758240782186887</v>
+        <v>0.3163870469997221</v>
       </c>
     </row>
     <row r="41">
@@ -1658,13 +1658,13 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>123</v>
+        <v>43</v>
       </c>
       <c r="C41" t="n">
-        <v>0.15188</v>
+        <v>0.08885</v>
       </c>
       <c r="D41" t="n">
-        <v>0.1822710569105691</v>
+        <v>0.1496648837209302</v>
       </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
@@ -1679,7 +1679,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>0.09987169756249363</v>
+        <v>0.6732029261945247</v>
       </c>
     </row>
     <row r="42">
@@ -1689,13 +1689,13 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>119</v>
+        <v>43</v>
       </c>
       <c r="C42" t="n">
-        <v>0.17647</v>
+        <v>0.11813</v>
       </c>
       <c r="D42" t="n">
-        <v>0.2028892436974789</v>
+        <v>0.1795002325581395</v>
       </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr"/>
@@ -1707,13 +1707,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>223</v>
+        <v>64</v>
       </c>
       <c r="C43" t="n">
-        <v>0.17287</v>
+        <v>0.213485</v>
       </c>
       <c r="D43" t="n">
-        <v>0.2111335874439462</v>
+        <v>0.22816484375</v>
       </c>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
@@ -1725,13 +1725,13 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>211</v>
+        <v>64</v>
       </c>
       <c r="C44" t="n">
-        <v>0.20263</v>
+        <v>0.228195</v>
       </c>
       <c r="D44" t="n">
-        <v>0.2372336018957346</v>
+        <v>0.2574215625</v>
       </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr"/>
@@ -2284,7 +2284,7 @@
         </is>
       </c>
       <c r="K62" t="n">
-        <v>0.008354066944748365</v>
+        <v>0.06709421409057292</v>
       </c>
     </row>
     <row r="63">
@@ -2294,13 +2294,13 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>118</v>
+        <v>43</v>
       </c>
       <c r="C63" t="n">
-        <v>3.999054291674237</v>
+        <v>4.109196794800181</v>
       </c>
       <c r="D63" t="n">
-        <v>4.526129390210736</v>
+        <v>5.364312607098492</v>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
@@ -2315,7 +2315,7 @@
         </is>
       </c>
       <c r="K63" t="n">
-        <v>0.0003568037253399673</v>
+        <v>0.01028302547111764</v>
       </c>
     </row>
     <row r="64">
@@ -2325,13 +2325,13 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>116</v>
+        <v>43</v>
       </c>
       <c r="C64" t="n">
-        <v>5.251924090162097</v>
+        <v>6.641933132185906</v>
       </c>
       <c r="D64" t="n">
-        <v>6.85399604891145</v>
+        <v>7.503748410889711</v>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr"/>
@@ -2343,13 +2343,13 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>210</v>
+        <v>62</v>
       </c>
       <c r="C65" t="n">
-        <v>2.631191964507098</v>
+        <v>4.106067773864563</v>
       </c>
       <c r="D65" t="n">
-        <v>3.532269244341498</v>
+        <v>4.788068887826513</v>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
@@ -2361,13 +2361,13 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>199</v>
+        <v>62</v>
       </c>
       <c r="C66" t="n">
-        <v>4.346864418261165</v>
+        <v>5.453969022321848</v>
       </c>
       <c r="D66" t="n">
-        <v>6.297895604967779</v>
+        <v>6.938116235074241</v>
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>0.1643488033433622</v>
+        <v>0.1306678087810564</v>
       </c>
     </row>
     <row r="19">
@@ -2991,13 +2991,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>110</v>
+        <v>43</v>
       </c>
       <c r="C19" t="n">
-        <v>0.5594303558360441</v>
+        <v>0.4284652106638905</v>
       </c>
       <c r="D19" t="n">
-        <v>0.6484981846936935</v>
+        <v>0.4905590988639374</v>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
@@ -3012,7 +3012,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>1.021692979439843e-05</v>
+        <v>0.006920243027168507</v>
       </c>
     </row>
     <row r="20">
@@ -3022,13 +3022,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>108</v>
+        <v>43</v>
       </c>
       <c r="C20" t="n">
-        <v>0.6573297656053722</v>
+        <v>0.4955263241944502</v>
       </c>
       <c r="D20" t="n">
-        <v>0.7088828450853494</v>
+        <v>0.5766951214543475</v>
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
@@ -3040,13 +3040,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>173</v>
+        <v>65</v>
       </c>
       <c r="C21" t="n">
-        <v>0.5541002514810333</v>
+        <v>0.5155670417103815</v>
       </c>
       <c r="D21" t="n">
-        <v>0.6239427351686871</v>
+        <v>0.5290488770317441</v>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
@@ -3058,13 +3058,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>152</v>
+        <v>65</v>
       </c>
       <c r="C22" t="n">
-        <v>0.763419027443043</v>
+        <v>0.6436724836308044</v>
       </c>
       <c r="D22" t="n">
-        <v>0.7674911636671264</v>
+        <v>0.691916063751258</v>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
@@ -3611,7 +3611,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>0.1135565290103986</v>
+        <v>0.3599067461079412</v>
       </c>
     </row>
     <row r="41">
@@ -3621,13 +3621,13 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>123</v>
+        <v>43</v>
       </c>
       <c r="C41" t="n">
-        <v>0.1051</v>
+        <v>0.0742</v>
       </c>
       <c r="D41" t="n">
-        <v>0.1377243902439024</v>
+        <v>0.1107767441860465</v>
       </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
@@ -3642,7 +3642,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>0.008056837686683409</v>
+        <v>0.3112026392410824</v>
       </c>
     </row>
     <row r="42">
@@ -3652,13 +3652,13 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>119</v>
+        <v>43</v>
       </c>
       <c r="C42" t="n">
-        <v>0.1187</v>
+        <v>0.0822</v>
       </c>
       <c r="D42" t="n">
-        <v>0.1654789915966387</v>
+        <v>0.1370093023255814</v>
       </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr"/>
@@ -3670,13 +3670,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>223</v>
+        <v>64</v>
       </c>
       <c r="C43" t="n">
-        <v>0.1176</v>
+        <v>0.1388</v>
       </c>
       <c r="D43" t="n">
-        <v>0.1602825112107623</v>
+        <v>0.174315625</v>
       </c>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
@@ -3688,13 +3688,13 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>211</v>
+        <v>64</v>
       </c>
       <c r="C44" t="n">
-        <v>0.155</v>
+        <v>0.16985</v>
       </c>
       <c r="D44" t="n">
-        <v>0.20840663507109</v>
+        <v>0.206315625</v>
       </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr"/>
@@ -4247,7 +4247,7 @@
         </is>
       </c>
       <c r="K62" t="n">
-        <v>0.1930399856579045</v>
+        <v>0.1373948258558008</v>
       </c>
     </row>
     <row r="63">
@@ -4257,13 +4257,13 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>108</v>
+        <v>43</v>
       </c>
       <c r="C63" t="n">
-        <v>0.6758214353450924</v>
+        <v>0.3857487965936796</v>
       </c>
       <c r="D63" t="n">
-        <v>0.645551442656028</v>
+        <v>0.4905670839875907</v>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
@@ -4278,7 +4278,7 @@
         </is>
       </c>
       <c r="K63" t="n">
-        <v>0.02107195494008832</v>
+        <v>0.01568164077814243</v>
       </c>
     </row>
     <row r="64">
@@ -4288,13 +4288,13 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>106</v>
+        <v>43</v>
       </c>
       <c r="C64" t="n">
-        <v>0.7366542149192417</v>
+        <v>0.6690443216615186</v>
       </c>
       <c r="D64" t="n">
-        <v>0.7191758079789841</v>
+        <v>0.6372987835990079</v>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr"/>
@@ -4306,13 +4306,13 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>163</v>
+        <v>62</v>
       </c>
       <c r="C65" t="n">
-        <v>0.5606030765555332</v>
+        <v>0.4154048678853915</v>
       </c>
       <c r="D65" t="n">
-        <v>0.5729076666951721</v>
+        <v>0.4708173574138831</v>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
@@ -4324,13 +4324,13 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>141</v>
+        <v>62</v>
       </c>
       <c r="C66" t="n">
-        <v>0.6673666861092722</v>
+        <v>0.6487075673530464</v>
       </c>
       <c r="D66" t="n">
-        <v>0.6710039905688603</v>
+        <v>0.645408287195066</v>
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
@@ -4944,7 +4944,7 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>0.01410870956425703</v>
+        <v>0.06709421409057292</v>
       </c>
     </row>
     <row r="19">
@@ -4954,13 +4954,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>123</v>
+        <v>43</v>
       </c>
       <c r="C19" t="n">
-        <v>3.922850941784398</v>
+        <v>4.109196794800181</v>
       </c>
       <c r="D19" t="n">
-        <v>4.35551863994824</v>
+        <v>5.364312607098492</v>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
@@ -4975,7 +4975,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>0.001090740331685134</v>
+        <v>0.0152689620777363</v>
       </c>
     </row>
     <row r="20">
@@ -4985,13 +4985,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>121</v>
+        <v>43</v>
       </c>
       <c r="C20" t="n">
-        <v>4.986877863043946</v>
+        <v>6.641933132185906</v>
       </c>
       <c r="D20" t="n">
-        <v>6.586981241961363</v>
+        <v>7.503748410889711</v>
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
@@ -5003,13 +5003,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>224</v>
+        <v>65</v>
       </c>
       <c r="C21" t="n">
-        <v>2.61261369468424</v>
+        <v>4.068351377792434</v>
       </c>
       <c r="D21" t="n">
-        <v>3.432583044683507</v>
+        <v>4.743535440975451</v>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
@@ -5021,13 +5021,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>213</v>
+        <v>65</v>
       </c>
       <c r="C22" t="n">
-        <v>3.866032886572921</v>
+        <v>4.526670375149739</v>
       </c>
       <c r="D22" t="n">
-        <v>5.985596104173117</v>
+        <v>6.763066931429598</v>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
@@ -5574,7 +5574,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>0.5690790091993174</v>
+        <v>0.8089074060398543</v>
       </c>
     </row>
     <row r="41">
@@ -5584,13 +5584,13 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>123</v>
+        <v>43</v>
       </c>
       <c r="C41" t="n">
-        <v>0.6394</v>
+        <v>0.6291</v>
       </c>
       <c r="D41" t="n">
-        <v>0.7480934959349592</v>
+        <v>0.7308139534883721</v>
       </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
@@ -5605,7 +5605,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>0.04315707690858427</v>
+        <v>0.5418627053816409</v>
       </c>
     </row>
     <row r="42">
@@ -5615,13 +5615,13 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>119</v>
+        <v>43</v>
       </c>
       <c r="C42" t="n">
-        <v>0.6656</v>
+        <v>0.6263</v>
       </c>
       <c r="D42" t="n">
-        <v>1.849619327731092</v>
+        <v>0.8450372093023257</v>
       </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr"/>
@@ -5633,13 +5633,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>223</v>
+        <v>64</v>
       </c>
       <c r="C43" t="n">
-        <v>0.6539</v>
+        <v>0.67605</v>
       </c>
       <c r="D43" t="n">
-        <v>0.9860403587443948</v>
+        <v>0.7172171875</v>
       </c>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
@@ -5651,13 +5651,13 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>211</v>
+        <v>64</v>
       </c>
       <c r="C44" t="n">
-        <v>0.7023</v>
+        <v>0.6738999999999999</v>
       </c>
       <c r="D44" t="n">
-        <v>2.372728436018957</v>
+        <v>1.3105671875</v>
       </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr"/>
@@ -6210,7 +6210,7 @@
         </is>
       </c>
       <c r="K62" t="n">
-        <v>0.00315367822989782</v>
+        <v>0.004779371916854929</v>
       </c>
     </row>
     <row r="63">
@@ -6220,13 +6220,13 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>83</v>
+        <v>43</v>
       </c>
       <c r="C63" t="n">
         <v>0</v>
       </c>
       <c r="D63" t="n">
-        <v>0.1570639701663798</v>
+        <v>0.1532530454042082</v>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
@@ -6241,7 +6241,7 @@
         </is>
       </c>
       <c r="K63" t="n">
-        <v>6.168068590191524e-10</v>
+        <v>6.816821218303963e-05</v>
       </c>
     </row>
     <row r="64">
@@ -6251,13 +6251,13 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C64" t="n">
-        <v>0.25</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="D64" t="n">
-        <v>0.272424684159378</v>
+        <v>0.3033637873754153</v>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr"/>
@@ -6269,13 +6269,13 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>127</v>
+        <v>62</v>
       </c>
       <c r="C65" t="n">
-        <v>0</v>
+        <v>0.0625</v>
       </c>
       <c r="D65" t="n">
-        <v>0.09211192350956131</v>
+        <v>0.1353014592933948</v>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
@@ -6287,13 +6287,13 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="C66" t="n">
         <v>0.25</v>
       </c>
       <c r="D66" t="n">
-        <v>0.2448809523809524</v>
+        <v>0.2586213517665131</v>
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
@@ -6907,7 +6907,7 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>0.1840751043955202</v>
+        <v>0.1373948258558008</v>
       </c>
     </row>
     <row r="19">
@@ -6917,13 +6917,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>110</v>
+        <v>43</v>
       </c>
       <c r="C19" t="n">
-        <v>0.6758214353450924</v>
+        <v>0.3857487965936796</v>
       </c>
       <c r="D19" t="n">
-        <v>0.6418688027696773</v>
+        <v>0.4905670839875907</v>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
@@ -6938,7 +6938,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>0.0132086937487541</v>
+        <v>0.01450284555131598</v>
       </c>
     </row>
     <row r="20">
@@ -6948,13 +6948,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>108</v>
+        <v>43</v>
       </c>
       <c r="C20" t="n">
-        <v>0.7366542149192417</v>
+        <v>0.6690443216615186</v>
       </c>
       <c r="D20" t="n">
-        <v>0.7167631455920301</v>
+        <v>0.6372987835990079</v>
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
@@ -6966,13 +6966,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>173</v>
+        <v>65</v>
       </c>
       <c r="C21" t="n">
-        <v>0.5731958394598844</v>
+        <v>0.4219521093748407</v>
       </c>
       <c r="D21" t="n">
-        <v>0.5863135694980639</v>
+        <v>0.473851380211333</v>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
@@ -6984,13 +6984,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>152</v>
+        <v>65</v>
       </c>
       <c r="C22" t="n">
-        <v>0.6777660562758083</v>
+        <v>0.6376628028208489</v>
       </c>
       <c r="D22" t="n">
-        <v>0.690619828760061</v>
+        <v>0.6440831151768942</v>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
@@ -7543,7 +7543,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>0.9930652022298012</v>
+        <v>0.9862180395120353</v>
       </c>
     </row>
     <row r="41">
@@ -7553,13 +7553,13 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>118</v>
+        <v>43</v>
       </c>
       <c r="C41" t="n">
-        <v>39.6272258423655</v>
+        <v>81.10617979073703</v>
       </c>
       <c r="D41" t="n">
-        <v>544.0751419339549</v>
+        <v>1272.711691675059</v>
       </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
@@ -7574,7 +7574,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>0.882241935173067</v>
+        <v>0.8906921514029046</v>
       </c>
     </row>
     <row r="42">
@@ -7584,13 +7584,13 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>116</v>
+        <v>43</v>
       </c>
       <c r="C42" t="n">
-        <v>37.72743858643629</v>
+        <v>87.69343443488347</v>
       </c>
       <c r="D42" t="n">
-        <v>665.3533717472737</v>
+        <v>1557.046404031143</v>
       </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr"/>
@@ -7602,13 +7602,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>210</v>
+        <v>62</v>
       </c>
       <c r="C43" t="n">
-        <v>25.42700294927524</v>
+        <v>55.32556858238002</v>
       </c>
       <c r="D43" t="n">
-        <v>301.3346448142449</v>
+        <v>319.2588292097612</v>
       </c>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
@@ -7620,13 +7620,13 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>199</v>
+        <v>62</v>
       </c>
       <c r="C44" t="n">
-        <v>20.26929003840828</v>
+        <v>46.64930600704498</v>
       </c>
       <c r="D44" t="n">
-        <v>388.0001654743568</v>
+        <v>657.390347836143</v>
       </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr"/>
@@ -8173,7 +8173,7 @@
         </is>
       </c>
       <c r="K62" t="n">
-        <v>0.1843066317127091</v>
+        <v>0.3163870469997221</v>
       </c>
     </row>
     <row r="63">
@@ -8183,13 +8183,13 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>118</v>
+        <v>43</v>
       </c>
       <c r="C63" t="n">
-        <v>0.147465</v>
+        <v>0.08885</v>
       </c>
       <c r="D63" t="n">
-        <v>0.1807242372881356</v>
+        <v>0.1496648837209302</v>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
@@ -8204,7 +8204,7 @@
         </is>
       </c>
       <c r="K63" t="n">
-        <v>0.05284520049655592</v>
+        <v>0.6375803044151374</v>
       </c>
     </row>
     <row r="64">
@@ -8214,13 +8214,13 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>114</v>
+        <v>43</v>
       </c>
       <c r="C64" t="n">
-        <v>0.16876</v>
+        <v>0.11813</v>
       </c>
       <c r="D64" t="n">
-        <v>0.2013262280701754</v>
+        <v>0.1795002325581395</v>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr"/>
@@ -8232,13 +8232,13 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>209</v>
+        <v>61</v>
       </c>
       <c r="C65" t="n">
-        <v>0.17018</v>
+        <v>0.22467</v>
       </c>
       <c r="D65" t="n">
-        <v>0.2073253110047847</v>
+        <v>0.2312613114754098</v>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
@@ -8250,13 +8250,13 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>197</v>
+        <v>61</v>
       </c>
       <c r="C66" t="n">
-        <v>0.20353</v>
+        <v>0.25077</v>
       </c>
       <c r="D66" t="n">
-        <v>0.2385574111675127</v>
+        <v>0.2623408196721311</v>
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
@@ -8870,7 +8870,7 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>0.00315367822989782</v>
+        <v>0.004779371916854929</v>
       </c>
     </row>
     <row r="19">
@@ -8880,13 +8880,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>83</v>
+        <v>43</v>
       </c>
       <c r="C19" t="n">
         <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>0.1570639701663798</v>
+        <v>0.1532530454042082</v>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
@@ -8901,7 +8901,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>2.056424389735719e-09</v>
+        <v>0.0001376337485387679</v>
       </c>
     </row>
     <row r="20">
@@ -8911,13 +8911,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C20" t="n">
-        <v>0.25</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="D20" t="n">
-        <v>0.272424684159378</v>
+        <v>0.3033637873754153</v>
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
@@ -8929,13 +8929,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>131</v>
+        <v>65</v>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>0.0625</v>
       </c>
       <c r="D21" t="n">
-        <v>0.09638767720828791</v>
+        <v>0.1432051282051282</v>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
@@ -8947,13 +8947,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="C22" t="n">
         <v>0.25</v>
       </c>
       <c r="D22" t="n">
-        <v>0.2440310846560847</v>
+        <v>0.2598717948717948</v>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
@@ -9506,7 +9506,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>0.1699713907690759</v>
+        <v>0.1306678087810564</v>
       </c>
     </row>
     <row r="41">
@@ -9516,13 +9516,13 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>108</v>
+        <v>43</v>
       </c>
       <c r="C41" t="n">
-        <v>0.5527241890383854</v>
+        <v>0.4284652106638905</v>
       </c>
       <c r="D41" t="n">
-        <v>0.6460681267736677</v>
+        <v>0.4905590988639374</v>
       </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
@@ -9537,7 +9537,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>8.035760071483031e-06</v>
+        <v>0.006409135806997244</v>
       </c>
     </row>
     <row r="42">
@@ -9547,13 +9547,13 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>106</v>
+        <v>43</v>
       </c>
       <c r="C42" t="n">
-        <v>0.6470023713560547</v>
+        <v>0.4955263241944502</v>
       </c>
       <c r="D42" t="n">
-        <v>0.7066517551414869</v>
+        <v>0.5766951214543475</v>
       </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr"/>
@@ -9565,13 +9565,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>163</v>
+        <v>62</v>
       </c>
       <c r="C43" t="n">
-        <v>0.5374036280348762</v>
+        <v>0.5053810014781956</v>
       </c>
       <c r="D43" t="n">
-        <v>0.6053395245408076</v>
+        <v>0.5203904752857982</v>
       </c>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
@@ -9583,13 +9583,13 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>141</v>
+        <v>62</v>
       </c>
       <c r="C44" t="n">
-        <v>0.7481444823317237</v>
+        <v>0.6432510769645133</v>
       </c>
       <c r="D44" t="n">
-        <v>0.7543155170341934</v>
+        <v>0.6909539601300555</v>
       </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr"/>
@@ -10136,7 +10136,7 @@
         </is>
       </c>
       <c r="K62" t="n">
-        <v>0.1289165535613832</v>
+        <v>0.3599067461079412</v>
       </c>
     </row>
     <row r="63">
@@ -10146,13 +10146,13 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>118</v>
+        <v>43</v>
       </c>
       <c r="C63" t="n">
-        <v>0.10495</v>
+        <v>0.0742</v>
       </c>
       <c r="D63" t="n">
-        <v>0.1348822033898305</v>
+        <v>0.1107767441860465</v>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
@@ -10167,7 +10167,7 @@
         </is>
       </c>
       <c r="K63" t="n">
-        <v>0.006416257180362809</v>
+        <v>0.2962120262353095</v>
       </c>
     </row>
     <row r="64">
@@ -10177,13 +10177,13 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>114</v>
+        <v>43</v>
       </c>
       <c r="C64" t="n">
-        <v>0.1156</v>
+        <v>0.0822</v>
       </c>
       <c r="D64" t="n">
-        <v>0.1625649122807018</v>
+        <v>0.1370093023255814</v>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr"/>
@@ -10195,13 +10195,13 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>209</v>
+        <v>61</v>
       </c>
       <c r="C65" t="n">
-        <v>0.1123</v>
+        <v>0.1494</v>
       </c>
       <c r="D65" t="n">
-        <v>0.1576842105263158</v>
+        <v>0.1778803278688525</v>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
@@ -10213,13 +10213,13 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>197</v>
+        <v>61</v>
       </c>
       <c r="C66" t="n">
-        <v>0.155</v>
+        <v>0.1809</v>
       </c>
       <c r="D66" t="n">
-        <v>0.1946203045685279</v>
+        <v>0.2112131147540983</v>
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
@@ -10827,7 +10827,7 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>0.1758240782186887</v>
+        <v>0.3163870469997221</v>
       </c>
     </row>
     <row r="19">
@@ -10837,13 +10837,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>123</v>
+        <v>43</v>
       </c>
       <c r="C19" t="n">
-        <v>0.15188</v>
+        <v>0.08885</v>
       </c>
       <c r="D19" t="n">
-        <v>0.1822710569105691</v>
+        <v>0.1496648837209302</v>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
@@ -10858,7 +10858,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>0.09987169756249363</v>
+        <v>0.6732029261945247</v>
       </c>
     </row>
     <row r="20">
@@ -10868,13 +10868,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>119</v>
+        <v>43</v>
       </c>
       <c r="C20" t="n">
-        <v>0.17647</v>
+        <v>0.11813</v>
       </c>
       <c r="D20" t="n">
-        <v>0.2028892436974789</v>
+        <v>0.1795002325581395</v>
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
@@ -10886,13 +10886,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>223</v>
+        <v>64</v>
       </c>
       <c r="C21" t="n">
-        <v>0.17287</v>
+        <v>0.213485</v>
       </c>
       <c r="D21" t="n">
-        <v>0.2111335874439462</v>
+        <v>0.22816484375</v>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
@@ -10904,13 +10904,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>211</v>
+        <v>64</v>
       </c>
       <c r="C22" t="n">
-        <v>0.20263</v>
+        <v>0.228195</v>
       </c>
       <c r="D22" t="n">
-        <v>0.2372336018957346</v>
+        <v>0.2574215625</v>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
@@ -11463,7 +11463,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>0.008354066944748365</v>
+        <v>0.06709421409057292</v>
       </c>
     </row>
     <row r="41">
@@ -11473,13 +11473,13 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>118</v>
+        <v>43</v>
       </c>
       <c r="C41" t="n">
-        <v>3.999054291674237</v>
+        <v>4.109196794800181</v>
       </c>
       <c r="D41" t="n">
-        <v>4.526129390210736</v>
+        <v>5.364312607098492</v>
       </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
@@ -11494,7 +11494,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>0.0003568037253399673</v>
+        <v>0.01028302547111764</v>
       </c>
     </row>
     <row r="42">
@@ -11504,13 +11504,13 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>116</v>
+        <v>43</v>
       </c>
       <c r="C42" t="n">
-        <v>5.251924090162097</v>
+        <v>6.641933132185906</v>
       </c>
       <c r="D42" t="n">
-        <v>6.85399604891145</v>
+        <v>7.503748410889711</v>
       </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr"/>
@@ -11522,13 +11522,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>210</v>
+        <v>62</v>
       </c>
       <c r="C43" t="n">
-        <v>2.631191964507098</v>
+        <v>4.106067773864563</v>
       </c>
       <c r="D43" t="n">
-        <v>3.532269244341498</v>
+        <v>4.788068887826513</v>
       </c>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
@@ -11540,13 +11540,13 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>199</v>
+        <v>62</v>
       </c>
       <c r="C44" t="n">
-        <v>4.346864418261165</v>
+        <v>5.453969022321848</v>
       </c>
       <c r="D44" t="n">
-        <v>6.297895604967779</v>
+        <v>6.938116235074241</v>
       </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr"/>
@@ -12093,7 +12093,7 @@
         </is>
       </c>
       <c r="K62" t="n">
-        <v>0.5764125706003373</v>
+        <v>0.8089074060398543</v>
       </c>
     </row>
     <row r="63">
@@ -12103,13 +12103,13 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>118</v>
+        <v>43</v>
       </c>
       <c r="C63" t="n">
-        <v>0.63325</v>
+        <v>0.6291</v>
       </c>
       <c r="D63" t="n">
-        <v>0.7375330508474575</v>
+        <v>0.7308139534883721</v>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
@@ -12124,7 +12124,7 @@
         </is>
       </c>
       <c r="K63" t="n">
-        <v>0.07472351777010704</v>
+        <v>0.6467482960754847</v>
       </c>
     </row>
     <row r="64">
@@ -12134,13 +12134,13 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>114</v>
+        <v>43</v>
       </c>
       <c r="C64" t="n">
-        <v>0.6535</v>
+        <v>0.6263</v>
       </c>
       <c r="D64" t="n">
-        <v>1.884848245614035</v>
+        <v>0.8450372093023257</v>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr"/>
@@ -12152,13 +12152,13 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>209</v>
+        <v>61</v>
       </c>
       <c r="C65" t="n">
-        <v>0.651</v>
+        <v>0.6766</v>
       </c>
       <c r="D65" t="n">
-        <v>0.7368205741626794</v>
+        <v>0.7227032786885246</v>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
@@ -12170,13 +12170,13 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>197</v>
+        <v>61</v>
       </c>
       <c r="C66" t="n">
-        <v>0.6937</v>
+        <v>0.6703</v>
       </c>
       <c r="D66" t="n">
-        <v>1.131240101522843</v>
+        <v>1.340009836065574</v>
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
@@ -12784,7 +12784,7 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>0.1135565290103986</v>
+        <v>0.3599067461079412</v>
       </c>
     </row>
     <row r="19">
@@ -12794,13 +12794,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>123</v>
+        <v>43</v>
       </c>
       <c r="C19" t="n">
-        <v>0.1051</v>
+        <v>0.0742</v>
       </c>
       <c r="D19" t="n">
-        <v>0.1377243902439024</v>
+        <v>0.1107767441860465</v>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
@@ -12815,7 +12815,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>0.008056837686683409</v>
+        <v>0.3112026392410824</v>
       </c>
     </row>
     <row r="20">
@@ -12825,13 +12825,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>119</v>
+        <v>43</v>
       </c>
       <c r="C20" t="n">
-        <v>0.1187</v>
+        <v>0.0822</v>
       </c>
       <c r="D20" t="n">
-        <v>0.1654789915966387</v>
+        <v>0.1370093023255814</v>
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
@@ -12843,13 +12843,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>223</v>
+        <v>64</v>
       </c>
       <c r="C21" t="n">
-        <v>0.1176</v>
+        <v>0.1388</v>
       </c>
       <c r="D21" t="n">
-        <v>0.1602825112107623</v>
+        <v>0.174315625</v>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
@@ -12861,13 +12861,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>211</v>
+        <v>64</v>
       </c>
       <c r="C22" t="n">
-        <v>0.155</v>
+        <v>0.16985</v>
       </c>
       <c r="D22" t="n">
-        <v>0.20840663507109</v>
+        <v>0.206315625</v>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
@@ -13420,7 +13420,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>0.1930399856579045</v>
+        <v>0.1373948258558008</v>
       </c>
     </row>
     <row r="41">
@@ -13430,13 +13430,13 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>108</v>
+        <v>43</v>
       </c>
       <c r="C41" t="n">
-        <v>0.6758214353450924</v>
+        <v>0.3857487965936796</v>
       </c>
       <c r="D41" t="n">
-        <v>0.645551442656028</v>
+        <v>0.4905670839875907</v>
       </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
@@ -13451,7 +13451,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>0.02107195494008832</v>
+        <v>0.01568164077814243</v>
       </c>
     </row>
     <row r="42">
@@ -13461,13 +13461,13 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>106</v>
+        <v>43</v>
       </c>
       <c r="C42" t="n">
-        <v>0.7366542149192417</v>
+        <v>0.6690443216615186</v>
       </c>
       <c r="D42" t="n">
-        <v>0.7191758079789841</v>
+        <v>0.6372987835990079</v>
       </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr"/>
@@ -13479,13 +13479,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>163</v>
+        <v>62</v>
       </c>
       <c r="C43" t="n">
-        <v>0.5606030765555332</v>
+        <v>0.4154048678853915</v>
       </c>
       <c r="D43" t="n">
-        <v>0.5729076666951721</v>
+        <v>0.4708173574138831</v>
       </c>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
@@ -13497,13 +13497,13 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>141</v>
+        <v>62</v>
       </c>
       <c r="C44" t="n">
-        <v>0.6673666861092722</v>
+        <v>0.6487075673530464</v>
       </c>
       <c r="D44" t="n">
-        <v>0.6710039905688603</v>
+        <v>0.645408287195066</v>
       </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr"/>
@@ -14056,7 +14056,7 @@
         </is>
       </c>
       <c r="K62" t="n">
-        <v>0.9102312141258041</v>
+        <v>0.9892934350380885</v>
       </c>
     </row>
     <row r="63">
@@ -14066,13 +14066,13 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>118</v>
+        <v>42</v>
       </c>
       <c r="C63" t="n">
-        <v>34.6367835312451</v>
+        <v>82.27949530216745</v>
       </c>
       <c r="D63" t="n">
-        <v>537.3654466248075</v>
+        <v>1302.971719023794</v>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
@@ -14087,7 +14087,7 @@
         </is>
       </c>
       <c r="K63" t="n">
-        <v>0.9150858071534826</v>
+        <v>0.8558998054368265</v>
       </c>
     </row>
     <row r="64">
@@ -14097,13 +14097,13 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>119</v>
+        <v>42</v>
       </c>
       <c r="C64" t="n">
-        <v>33.95292213898919</v>
+        <v>88.47851396671578</v>
       </c>
       <c r="D64" t="n">
-        <v>646.6579122667524</v>
+        <v>1594.019582567449</v>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr"/>
@@ -14115,13 +14115,13 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>212</v>
+        <v>65</v>
       </c>
       <c r="C65" t="n">
-        <v>20.95279149208183</v>
+        <v>42.05024144982589</v>
       </c>
       <c r="D65" t="n">
-        <v>293.6190265121362</v>
+        <v>305.2020155903968</v>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
@@ -14133,13 +14133,13 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>213</v>
+        <v>65</v>
       </c>
       <c r="C66" t="n">
-        <v>16.67727831298509</v>
+        <v>39.91526560386543</v>
       </c>
       <c r="D66" t="n">
-        <v>362.7401690272649</v>
+        <v>627.511222150869</v>
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
@@ -14747,7 +14747,7 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>0.5690790091993174</v>
+        <v>0.8089074060398543</v>
       </c>
     </row>
     <row r="19">
@@ -14757,13 +14757,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>123</v>
+        <v>43</v>
       </c>
       <c r="C19" t="n">
-        <v>0.6394</v>
+        <v>0.6291</v>
       </c>
       <c r="D19" t="n">
-        <v>0.7480934959349592</v>
+        <v>0.7308139534883721</v>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
@@ -14778,7 +14778,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>0.04315707690858427</v>
+        <v>0.5418627053816409</v>
       </c>
     </row>
     <row r="20">
@@ -14788,13 +14788,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>119</v>
+        <v>43</v>
       </c>
       <c r="C20" t="n">
-        <v>0.6656</v>
+        <v>0.6263</v>
       </c>
       <c r="D20" t="n">
-        <v>1.849619327731092</v>
+        <v>0.8450372093023257</v>
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
@@ -14806,13 +14806,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>223</v>
+        <v>64</v>
       </c>
       <c r="C21" t="n">
-        <v>0.6539</v>
+        <v>0.67605</v>
       </c>
       <c r="D21" t="n">
-        <v>0.9860403587443948</v>
+        <v>0.7172171875</v>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
@@ -14824,13 +14824,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>211</v>
+        <v>64</v>
       </c>
       <c r="C22" t="n">
-        <v>0.7023</v>
+        <v>0.6738999999999999</v>
       </c>
       <c r="D22" t="n">
-        <v>2.372728436018957</v>
+        <v>1.3105671875</v>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
@@ -15383,7 +15383,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>0.00315367822989782</v>
+        <v>0.004779371916854929</v>
       </c>
     </row>
     <row r="41">
@@ -15393,13 +15393,13 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>83</v>
+        <v>43</v>
       </c>
       <c r="C41" t="n">
         <v>0</v>
       </c>
       <c r="D41" t="n">
-        <v>0.1570639701663798</v>
+        <v>0.1532530454042082</v>
       </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
@@ -15414,7 +15414,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>6.168068590191524e-10</v>
+        <v>6.816821218303963e-05</v>
       </c>
     </row>
     <row r="42">
@@ -15424,13 +15424,13 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C42" t="n">
-        <v>0.25</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="D42" t="n">
-        <v>0.272424684159378</v>
+        <v>0.3033637873754153</v>
       </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr"/>
@@ -15442,13 +15442,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>127</v>
+        <v>62</v>
       </c>
       <c r="C43" t="n">
-        <v>0</v>
+        <v>0.0625</v>
       </c>
       <c r="D43" t="n">
-        <v>0.09211192350956131</v>
+        <v>0.1353014592933948</v>
       </c>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
@@ -15460,13 +15460,13 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="C44" t="n">
         <v>0.25</v>
       </c>
       <c r="D44" t="n">
-        <v>0.2448809523809524</v>
+        <v>0.2586213517665131</v>
       </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr"/>
@@ -16019,7 +16019,7 @@
         </is>
       </c>
       <c r="K62" t="n">
-        <v>0.1882146432975397</v>
+        <v>0.1930354027430238</v>
       </c>
     </row>
     <row r="63">
@@ -16029,13 +16029,13 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>105</v>
+        <v>42</v>
       </c>
       <c r="C63" t="n">
-        <v>0.5558191599219442</v>
+        <v>0.4326044342266125</v>
       </c>
       <c r="D63" t="n">
-        <v>0.6456718528438683</v>
+        <v>0.4939146108377897</v>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
@@ -16050,7 +16050,7 @@
         </is>
       </c>
       <c r="K63" t="n">
-        <v>1.503389913975827e-05</v>
+        <v>0.006920243027168507</v>
       </c>
     </row>
     <row r="64">
@@ -16060,13 +16060,13 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>106</v>
+        <v>42</v>
       </c>
       <c r="C64" t="n">
-        <v>0.6470023713560547</v>
+        <v>0.4944849688972288</v>
       </c>
       <c r="D64" t="n">
-        <v>0.705160447046111</v>
+        <v>0.5673875556264958</v>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr"/>
@@ -16078,13 +16078,13 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>161</v>
+        <v>65</v>
       </c>
       <c r="C65" t="n">
-        <v>0.5541002514810333</v>
+        <v>0.5155670417103815</v>
       </c>
       <c r="D65" t="n">
-        <v>0.6239093426949556</v>
+        <v>0.5290488770317441</v>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
@@ -16096,13 +16096,13 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>152</v>
+        <v>65</v>
       </c>
       <c r="C66" t="n">
-        <v>0.763419027443043</v>
+        <v>0.6436724836308044</v>
       </c>
       <c r="D66" t="n">
-        <v>0.7674911636671264</v>
+        <v>0.691916063751258</v>
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>

</xml_diff>